<commit_message>
100 Mt + Net Zero
</commit_message>
<xml_diff>
--- a/data/data_analysis/carbon_costs.xlsx
+++ b/data/data_analysis/carbon_costs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\data\data_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2AE77E1-89B2-426E-BE5B-9E84213B9597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38929EB4-CDE0-4D64-B8BD-D5DEDF26DF96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{402A6D60-5D67-40F0-A8D8-2C5C69F3BFA7}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="57">
   <si>
     <t>High Baseline</t>
   </si>
@@ -189,6 +189,48 @@
   </si>
   <si>
     <t>Baseline</t>
+  </si>
+  <si>
+    <t>Costs in 2050</t>
+  </si>
+  <si>
+    <t>100 Mt CDR</t>
+  </si>
+  <si>
+    <t>500 Mt CDR</t>
+  </si>
+  <si>
+    <t>1500 Mt CDR</t>
+  </si>
+  <si>
+    <t>2400 Mt CDR</t>
+  </si>
+  <si>
+    <t>4000 Mt CDR</t>
+  </si>
+  <si>
+    <t>Effects of CDR Policy in 2050</t>
+  </si>
+  <si>
+    <t>500 Mt Baseline</t>
+  </si>
+  <si>
+    <t>500 Mt Procurement</t>
+  </si>
+  <si>
+    <t>500 Mt Tax Credit</t>
+  </si>
+  <si>
+    <t>500 Mt Innovation Policy</t>
+  </si>
+  <si>
+    <t>Positive CO2 emissions</t>
+  </si>
+  <si>
+    <t>Positive C emissions</t>
+  </si>
+  <si>
+    <t>Marginal Effectiveness</t>
   </si>
 </sst>
 </file>
@@ -3250,6 +3292,1490 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Cost of Achieving Net Zero 2050 in Various Scenarios</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.14532850060409117"/>
+          <c:y val="0.16429652554177632"/>
+          <c:w val="0.82557097029537962"/>
+          <c:h val="0.73203308979814574"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Total_Cost_Carbon!$R$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>CDR</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent5"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Total_Cost_Carbon!$S$3:$W$3</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>100 Mt CDR</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>500 Mt CDR</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1500 Mt CDR</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2400 Mt CDR</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4000 Mt CDR</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Total_Cost_Carbon!$S$4:$W$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>16.786343343126799</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>97.441209537122702</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>355.668987491883</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>608.06596042454896</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>947.56924633539904</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-37C6-4463-8E28-0E2438CE4F12}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Total_Cost_Carbon!$R$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>CO2 tax</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent3"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Total_Cost_Carbon!$S$3:$W$3</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>100 Mt CDR</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>500 Mt CDR</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1500 Mt CDR</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2400 Mt CDR</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4000 Mt CDR</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Total_Cost_Carbon!$S$5:$W$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>1292.5256363451399</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1271.7936232176701</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1200.7367084235</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>845.13026324293992</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-37C6-4463-8E28-0E2438CE4F12}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:overlap val="100"/>
+        <c:axId val="998777216"/>
+        <c:axId val="998791616"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="998777216"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="998791616"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="998791616"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" b="1"/>
+                  <a:t>Billion  USD/yr</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="2.1164021164021163E-2"/>
+              <c:y val="0.37020792913699702"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="998777216"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.7173226263383744"/>
+          <c:y val="0.16462306960242526"/>
+          <c:w val="0.24251156105486815"/>
+          <c:h val="8.7293538104897136E-2"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1050" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Cost of Achieving Net Zero 2050 by Policy Type</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.14532850060409117"/>
+          <c:y val="0.16429652554177632"/>
+          <c:w val="0.83615298087739021"/>
+          <c:h val="0.69474161098011766"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Total_Cost_Carbon!$R$9</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>CO2 tax</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent3"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Total_Cost_Carbon!$S$8:$V$8</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>500 Mt Baseline</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>500 Mt Procurement</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>500 Mt Tax Credit</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>500 Mt Innovation Policy</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Total_Cost_Carbon!$S$9:$V$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>1271.7936232176701</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1278.2202182165702</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1265.46770389566</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1261.2151652570799</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-DAF8-4736-82C8-0D3F102381A2}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Total_Cost_Carbon!$R$10</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>CDR</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent5"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Total_Cost_Carbon!$S$8:$V$8</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>500 Mt Baseline</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>500 Mt Procurement</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>500 Mt Tax Credit</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>500 Mt Innovation Policy</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Total_Cost_Carbon!$S$10:$V$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>97.441209537122702</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>97.8415030595731</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>95.558861633785511</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>83.465526403645498</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-DAF8-4736-82C8-0D3F102381A2}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:overlap val="100"/>
+        <c:axId val="998777216"/>
+        <c:axId val="998791616"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="998777216"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="998791616"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="998791616"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" b="1"/>
+                  <a:t>Billion USD/yr</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="2.1164021164021163E-2"/>
+              <c:y val="0.37020792913699702"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="998777216"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.7173226263383744"/>
+          <c:y val="0.16462306960242526"/>
+          <c:w val="0.24251156105486815"/>
+          <c:h val="8.7293538104897136E-2"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1050" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Moral Hazard of Increasing CDR</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.12513648293963256"/>
+          <c:y val="8.305736396855061E-2"/>
+          <c:w val="0.83286351706036732"/>
+          <c:h val="0.82245485258413076"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Total_Cost_Carbon!$Z$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Positive CO2 emissions</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="38100" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Total_Cost_Carbon!$AA$3:$AE$3</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1500</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2400</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Total_Cost_Carbon!$AA$4:$AE$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>3277.6882923332319</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3286.8508796772803</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3462.8793427374962</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3865.0223008479497</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4643.0507990947308</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-62FF-4D81-A351-67A8B52251F8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1043522208"/>
+        <c:axId val="1043512608"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1043522208"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Mt CDR/yr</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1043512608"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1043512608"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Mt</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> CO2 Emissions/yr</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1043522208"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -3450,6 +4976,126 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors6.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors7.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors8.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="332">
   <cs:axisTitle>
@@ -5954,6 +7600,1532 @@
         <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style6.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="297">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style7.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="297">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style8.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:valueAxis>
   <cs:wall>
@@ -6164,6 +9336,116 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>109537</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>600075</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="7" name="Chart 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F7858888-3724-6FB2-F95F-574FA0203F1D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>600075</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>176213</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="8" name="Chart 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F4767A67-470B-4588-B4F4-F91D239153DF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>109535</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>109535</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="9" name="Chart 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B9B2AFFF-92F9-99AB-0948-53C3F333BF02}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -7094,10 +10376,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0881DB2A-9C4C-46E9-980E-CFE273FA9402}">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:AE13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>37</v>
       </c>
@@ -7120,7 +10402,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>33</v>
       </c>
@@ -7142,8 +10424,29 @@
       <c r="G2" t="s">
         <v>36</v>
       </c>
+      <c r="S2" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z2">
+        <v>2050</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>44</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>46</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>47</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>48</v>
+      </c>
     </row>
-    <row r="3" spans="1:7" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:31" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="1"/>
       <c r="B3" t="s">
         <v>39</v>
@@ -7163,8 +10466,41 @@
       <c r="G3" t="s">
         <v>36</v>
       </c>
+      <c r="S3" t="s">
+        <v>44</v>
+      </c>
+      <c r="T3" t="s">
+        <v>45</v>
+      </c>
+      <c r="U3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V3" t="s">
+        <v>47</v>
+      </c>
+      <c r="W3" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA3">
+        <v>100</v>
+      </c>
+      <c r="AB3">
+        <v>500</v>
+      </c>
+      <c r="AC3">
+        <v>1500</v>
+      </c>
+      <c r="AD3">
+        <v>2400</v>
+      </c>
+      <c r="AE3">
+        <v>4000</v>
+      </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
@@ -7186,8 +10522,49 @@
       <c r="G4" t="s">
         <v>36</v>
       </c>
+      <c r="R4" t="s">
+        <v>35</v>
+      </c>
+      <c r="S4">
+        <v>16.786343343126799</v>
+      </c>
+      <c r="T4">
+        <v>97.441209537122702</v>
+      </c>
+      <c r="U4">
+        <v>355.668987491883</v>
+      </c>
+      <c r="V4">
+        <v>608.06596042454896</v>
+      </c>
+      <c r="W4">
+        <v>947.56924633539904</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>54</v>
+      </c>
+      <c r="AA4">
+        <f t="shared" ref="AA4:AD4" si="0">AA5*44/12</f>
+        <v>3277.6882923332319</v>
+      </c>
+      <c r="AB4">
+        <f t="shared" si="0"/>
+        <v>3286.8508796772803</v>
+      </c>
+      <c r="AC4">
+        <f t="shared" si="0"/>
+        <v>3462.8793427374962</v>
+      </c>
+      <c r="AD4">
+        <f t="shared" si="0"/>
+        <v>3865.0223008479497</v>
+      </c>
+      <c r="AE4">
+        <f>AE5*44/12</f>
+        <v>4643.0507990947308</v>
+      </c>
     </row>
-    <row r="5" spans="1:7" ht="18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:31" ht="18" x14ac:dyDescent="0.35">
       <c r="A5" s="1"/>
       <c r="B5" t="s">
         <v>39</v>
@@ -7207,8 +10584,44 @@
       <c r="G5" t="s">
         <v>36</v>
       </c>
+      <c r="R5" t="s">
+        <v>39</v>
+      </c>
+      <c r="S5">
+        <v>1292.5256363451399</v>
+      </c>
+      <c r="T5">
+        <v>1271.7936232176701</v>
+      </c>
+      <c r="U5">
+        <v>1200.7367084235</v>
+      </c>
+      <c r="V5">
+        <v>845.13026324293992</v>
+      </c>
+      <c r="W5">
+        <v>0</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA5">
+        <v>893.91498881815403</v>
+      </c>
+      <c r="AB5">
+        <v>896.41387627562199</v>
+      </c>
+      <c r="AC5">
+        <v>944.42163892840802</v>
+      </c>
+      <c r="AD5">
+        <v>1054.0969911403499</v>
+      </c>
+      <c r="AE5">
+        <v>1266.2865815712901</v>
+      </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
@@ -7230,8 +10643,27 @@
       <c r="G6" t="s">
         <v>36</v>
       </c>
+      <c r="Z6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB6">
+        <f>(AB4-AA4)/(AB3-AA3)</f>
+        <v>2.2906468360121154E-2</v>
+      </c>
+      <c r="AC6">
+        <f t="shared" ref="AC6:AE6" si="1">(AC4-AB4)/(AC3-AB3)</f>
+        <v>0.17602846306021594</v>
+      </c>
+      <c r="AD6">
+        <f t="shared" si="1"/>
+        <v>0.446825509011615</v>
+      </c>
+      <c r="AE6">
+        <f t="shared" si="1"/>
+        <v>0.48626781140423814</v>
+      </c>
     </row>
-    <row r="7" spans="1:7" ht="18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:31" ht="18" x14ac:dyDescent="0.35">
       <c r="A7" s="1"/>
       <c r="B7" t="s">
         <v>39</v>
@@ -7251,8 +10683,59 @@
       <c r="G7" t="s">
         <v>36</v>
       </c>
+      <c r="S7" t="s">
+        <v>49</v>
+      </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="S8" t="s">
+        <v>50</v>
+      </c>
+      <c r="T8" t="s">
+        <v>51</v>
+      </c>
+      <c r="U8" t="s">
+        <v>52</v>
+      </c>
+      <c r="V8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:31" ht="18" x14ac:dyDescent="0.35">
+      <c r="R9" t="s">
+        <v>39</v>
+      </c>
+      <c r="S9">
+        <v>1271.7936232176701</v>
+      </c>
+      <c r="T9">
+        <v>1278.2202182165702</v>
+      </c>
+      <c r="U9">
+        <v>1265.46770389566</v>
+      </c>
+      <c r="V9">
+        <v>1261.2151652570799</v>
+      </c>
+    </row>
+    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="R10" t="s">
+        <v>35</v>
+      </c>
+      <c r="S10">
+        <v>97.441209537122702</v>
+      </c>
+      <c r="T10">
+        <v>97.8415030595731</v>
+      </c>
+      <c r="U10">
+        <v>95.558861633785511</v>
+      </c>
+      <c r="V10">
+        <v>83.465526403645498</v>
+      </c>
+    </row>
+    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
         <v>42</v>
       </c>
@@ -7263,7 +10746,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:31" ht="18" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>39</v>
       </c>
@@ -7277,7 +10760,7 @@
         <v>1195154.91085111</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>35</v>
       </c>

</xml_diff>